<commit_message>
data(nzd): daily refresh 2026-10-01T10:45Z
</commit_message>
<xml_diff>
--- a/logs/nzd/raw/nzdm_ecp.xlsx
+++ b/logs/nzd/raw/nzdm_ecp.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cass.sharepoint.com/sites/TSYCapitalMarketsFundingStrategyandEngagement-FundingStrategyandEngagement/Shared Documents/Website data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B7F9C34-E9B5-4714-A493-714568D24E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{A3C507A8-94FD-429E-8821-D23EDD8338D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2CF60E1-3006-4E58-9823-FB4B1520ECA2}"/>
   <bookViews>
-    <workbookView xWindow="44880" yWindow="-465" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-195" yWindow="-16710" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Month_end" sheetId="11" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Month_end!$A$5:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Month_end!$A$6:$J$7</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>New Zealand Government Euro-Commercial Paper on Issue</t>
   </si>
@@ -59,7 +59,10 @@
     <t>* NZD equivalents are calculated by using end of month spot exchange rates. It is the rate published by the RBNZ (https://www.rbnz.govt.nz/statistics/b1) where possible, or the Bloomberg 14:00 rate</t>
   </si>
   <si>
-    <t>Published: 1 September 2026</t>
+    <t>Published: 1 October 2026</t>
+  </si>
+  <si>
+    <t>All data is based on settlement date (not trade date)</t>
   </si>
 </sst>
 </file>
@@ -72,7 +75,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,6 +102,11 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
@@ -144,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -190,6 +198,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -471,62 +482,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K131"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K133"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.42578125" customWidth="1"/>
+    <col min="1" max="1" width="13.81640625" customWidth="1"/>
+    <col min="2" max="2" width="13.81640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.54296875" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.453125" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="26.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="10">
-        <v>43951</v>
-      </c>
-      <c r="B6" s="14">
-        <v>530.52562846882142</v>
-      </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="6"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -534,14 +535,13 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="10">
-        <v>43982</v>
+        <v>43951</v>
       </c>
       <c r="B7" s="14">
-        <v>1004.3527325487668</v>
-      </c>
-      <c r="C7" s="7"/>
+        <v>530.52562846882142</v>
+      </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -550,12 +550,12 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
-        <v>44012</v>
+        <v>43982</v>
       </c>
       <c r="B8" s="14">
-        <v>1280.7345160286338</v>
+        <v>1004.3527325487668</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="2"/>
@@ -566,12 +566,12 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="10">
-        <v>44043</v>
+        <v>44012</v>
       </c>
       <c r="B9" s="14">
-        <v>1748.9926876585582</v>
+        <v>1280.7345160286338</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="2"/>
@@ -582,29 +582,28 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
-        <v>44074</v>
+        <v>44043</v>
       </c>
       <c r="B10" s="14">
-        <v>1837.8703564445782</v>
-      </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="13"/>
+        <v>1748.9926876585582</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="10">
-        <v>44104</v>
+        <v>44074</v>
       </c>
       <c r="B11" s="14">
-        <v>1131.3</v>
+        <v>1837.8703564445782</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13"/>
@@ -616,15 +615,15 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="10">
-        <v>44135</v>
-      </c>
-      <c r="B12" s="7">
-        <v>674.7</v>
-      </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="1"/>
+        <v>44104</v>
+      </c>
+      <c r="B12" s="14">
+        <v>1131.3</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="13"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -633,12 +632,12 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="10">
-        <v>44165</v>
+        <v>44135</v>
       </c>
       <c r="B13" s="7">
-        <v>1185.911092174407</v>
+        <v>674.7</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="1"/>
@@ -650,15 +649,15 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="10">
-        <v>44196</v>
+        <v>44165</v>
       </c>
       <c r="B14" s="7">
-        <v>1951.0170195101703</v>
+        <v>1185.911092174407</v>
       </c>
       <c r="C14" s="10"/>
-      <c r="D14" s="7"/>
+      <c r="D14" s="1"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -667,12 +666,12 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
-        <v>44227</v>
+        <v>44196</v>
       </c>
       <c r="B15" s="7">
-        <v>2050.78125</v>
+        <v>1951.0170195101703</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="7"/>
@@ -684,12 +683,12 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
-        <v>44255</v>
+        <v>44227</v>
       </c>
       <c r="B16" s="7">
-        <v>1081.7798339910191</v>
+        <v>2050.78125</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="7"/>
@@ -701,15 +700,15 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="10">
-        <v>44286</v>
+        <v>44255</v>
       </c>
       <c r="B17" s="7">
-        <v>1709.8297324366863</v>
+        <v>1081.7798339910191</v>
       </c>
       <c r="C17" s="10"/>
-      <c r="D17" s="1"/>
+      <c r="D17" s="7"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -718,15 +717,15 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="10">
-        <v>44316</v>
+        <v>44286</v>
       </c>
       <c r="B18" s="7">
-        <v>1510.2</v>
+        <v>1709.8297324366863</v>
       </c>
       <c r="C18" s="10"/>
-      <c r="D18" s="7"/>
+      <c r="D18" s="1"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -735,12 +734,12 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="10">
-        <v>44347</v>
+        <v>44316</v>
       </c>
       <c r="B19" s="7">
-        <v>1620.2</v>
+        <v>1510.2</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="7"/>
@@ -752,12 +751,12 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="10">
-        <v>44377</v>
+        <v>44347</v>
       </c>
       <c r="B20" s="7">
-        <v>1331.809088310946</v>
+        <v>1620.2</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="7"/>
@@ -769,15 +768,15 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="10">
-        <v>44408</v>
+        <v>44377</v>
       </c>
       <c r="B21" s="7">
-        <v>1674</v>
+        <v>1331.809088310946</v>
       </c>
       <c r="C21" s="10"/>
-      <c r="D21" s="1"/>
+      <c r="D21" s="7"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -786,29 +785,29 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="10">
-        <v>44439</v>
+        <v>44408</v>
       </c>
       <c r="B22" s="7">
-        <v>1774.8363222317109</v>
+        <v>1674</v>
       </c>
       <c r="C22" s="10"/>
-      <c r="D22" s="7"/>
+      <c r="D22" s="1"/>
       <c r="E22" s="2"/>
-      <c r="F22" s="5"/>
+      <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="10">
-        <v>44469</v>
+        <v>44439</v>
       </c>
       <c r="B23" s="7">
-        <v>1774.8036077974978</v>
+        <v>1774.8363222317109</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="7"/>
@@ -820,12 +819,12 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="10">
-        <v>44500</v>
+        <v>44469</v>
       </c>
       <c r="B24" s="7">
-        <v>1810.5849582172702</v>
+        <v>1774.8036077974978</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="7"/>
@@ -837,29 +836,29 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="10">
-        <v>44530</v>
+        <v>44500</v>
       </c>
       <c r="B25" s="7">
-        <v>1396.8462390584452</v>
+        <v>1810.5849582172702</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="7"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
+      <c r="F25" s="5"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="10">
-        <v>44561</v>
+        <v>44530</v>
       </c>
       <c r="B26" s="7">
-        <v>1653.9812646370021</v>
+        <v>1396.8462390584452</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="7"/>
@@ -871,12 +870,12 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="10">
-        <v>44592</v>
+        <v>44561</v>
       </c>
       <c r="B27" s="7">
-        <v>2314.3904674610453</v>
+        <v>1653.9812646370021</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="7"/>
@@ -888,12 +887,12 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="10">
-        <v>44620</v>
+        <v>44592</v>
       </c>
       <c r="B28" s="7">
-        <v>2481.3153961136022</v>
+        <v>2314.3904674610453</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="7"/>
@@ -905,15 +904,15 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="10">
-        <v>44651</v>
+        <v>44620</v>
       </c>
       <c r="B29" s="7">
-        <v>1727.5985663082438</v>
+        <v>2481.3153961136022</v>
       </c>
       <c r="C29" s="10"/>
-      <c r="D29" s="1"/>
+      <c r="D29" s="7"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
@@ -922,12 +921,12 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="10">
-        <v>44681</v>
+        <v>44651</v>
       </c>
       <c r="B30" s="7">
-        <v>1283.8253382533826</v>
+        <v>1727.5985663082438</v>
       </c>
       <c r="C30" s="10"/>
       <c r="D30" s="1"/>
@@ -939,12 +938,12 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="10">
-        <v>44712</v>
+        <v>44681</v>
       </c>
       <c r="B31" s="7">
-        <v>1592.4</v>
+        <v>1283.8253382533826</v>
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="1"/>
@@ -956,12 +955,12 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="10">
-        <v>44742</v>
+        <v>44712</v>
       </c>
       <c r="B32" s="7">
-        <v>1392.1</v>
+        <v>1592.4</v>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="1"/>
@@ -973,12 +972,12 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="10">
-        <v>44773</v>
+        <v>44742</v>
       </c>
       <c r="B33" s="7">
-        <v>1612.3907863383638</v>
+        <v>1392.1</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="1"/>
@@ -990,12 +989,12 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="10">
-        <v>44804</v>
+        <v>44773</v>
       </c>
       <c r="B34" s="7">
-        <v>1574</v>
+        <v>1612.3907863383638</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="1"/>
@@ -1007,12 +1006,12 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="10">
-        <v>44834</v>
+        <v>44804</v>
       </c>
       <c r="B35" s="7">
-        <v>1327.6</v>
+        <v>1574</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="1"/>
@@ -1024,12 +1023,12 @@
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="10">
-        <v>44865</v>
+        <v>44834</v>
       </c>
       <c r="B36" s="7">
-        <v>1406.2</v>
+        <v>1327.6</v>
       </c>
       <c r="C36" s="10"/>
       <c r="D36" s="1"/>
@@ -1041,12 +1040,12 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="10">
-        <v>44895</v>
+        <v>44865</v>
       </c>
       <c r="B37" s="7">
-        <v>1752.1</v>
+        <v>1406.2</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="1"/>
@@ -1058,53 +1057,53 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="10">
+        <v>44895</v>
+      </c>
+      <c r="B38" s="7">
+        <v>1752.1</v>
+      </c>
+      <c r="C38" s="10"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" s="10">
         <v>44926</v>
       </c>
-      <c r="B38" s="7">
+      <c r="B39" s="7">
         <v>1419.002975712843</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="10">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A40" s="10">
         <v>44957</v>
       </c>
-      <c r="B39" s="7">
+      <c r="B40" s="7">
         <v>1277.0562770562769</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="10">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41" s="10">
         <v>44985</v>
       </c>
-      <c r="B40" s="7">
+      <c r="B41" s="7">
         <v>2061.1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="10">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A42" s="10">
         <v>45016</v>
       </c>
-      <c r="B41" s="7">
+      <c r="B42" s="7">
         <v>1872.5</v>
-      </c>
-      <c r="C41" s="10"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="10">
-        <v>45046</v>
-      </c>
-      <c r="B42" s="7">
-        <v>1803.1189083820661</v>
       </c>
       <c r="C42" s="10"/>
       <c r="D42" s="7"/>
@@ -1116,12 +1115,12 @@
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="10">
-        <v>45077</v>
+        <v>45046</v>
       </c>
       <c r="B43" s="7">
-        <v>2102.2019110926462</v>
+        <v>1803.1189083820661</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="7"/>
@@ -1133,12 +1132,12 @@
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="10">
-        <v>45107</v>
+        <v>45077</v>
       </c>
       <c r="B44" s="7">
-        <v>1938.7497693891921</v>
+        <v>2102.2019110926462</v>
       </c>
       <c r="C44" s="10"/>
       <c r="D44" s="7"/>
@@ -1150,12 +1149,12 @@
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
-        <v>45138</v>
+        <v>45107</v>
       </c>
       <c r="B45" s="7">
-        <v>2128.8235077088689</v>
+        <v>1938.7497693891921</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="7"/>
@@ -1167,12 +1166,12 @@
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="10">
-        <v>45169</v>
+        <v>45138</v>
       </c>
       <c r="B46" s="7">
-        <v>2332.283486358695</v>
+        <v>2128.8235077088689</v>
       </c>
       <c r="C46" s="10"/>
       <c r="D46" s="7"/>
@@ -1184,12 +1183,12 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="10">
-        <v>45199</v>
+        <v>45169</v>
       </c>
       <c r="B47" s="7">
-        <v>3046.1311663080469</v>
+        <v>2332.283486358695</v>
       </c>
       <c r="C47" s="10"/>
       <c r="D47" s="7"/>
@@ -1201,12 +1200,12 @@
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="10">
-        <v>45230</v>
+        <v>45199</v>
       </c>
       <c r="B48" s="7">
-        <v>4402.570739501195</v>
+        <v>3046.1311663080469</v>
       </c>
       <c r="C48" s="10"/>
       <c r="D48" s="7"/>
@@ -1218,12 +1217,12 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="10">
-        <v>45260</v>
+        <v>45230</v>
       </c>
       <c r="B49" s="7">
-        <v>6769.1954608021688</v>
+        <v>4402.570739501195</v>
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="7"/>
@@ -1235,12 +1234,12 @@
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="10">
-        <v>45291</v>
+        <v>45260</v>
       </c>
       <c r="B50" s="7">
-        <v>7836.8620431861318</v>
+        <v>6769.1954608021688</v>
       </c>
       <c r="C50" s="10"/>
       <c r="D50" s="7"/>
@@ -1252,12 +1251,12 @@
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="10">
-        <v>45322</v>
+        <v>45291</v>
       </c>
       <c r="B51" s="7">
-        <v>9712.2000000000007</v>
+        <v>7836.8620431861318</v>
       </c>
       <c r="C51" s="10"/>
       <c r="D51" s="7"/>
@@ -1269,12 +1268,12 @@
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="10">
-        <v>45351</v>
+        <v>45322</v>
       </c>
       <c r="B52" s="7">
-        <v>9546.6869690003168</v>
+        <v>9712.2000000000007</v>
       </c>
       <c r="C52" s="10"/>
       <c r="D52" s="7"/>
@@ -1286,12 +1285,12 @@
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="10">
-        <v>45382</v>
+        <v>45351</v>
       </c>
       <c r="B53" s="7">
-        <v>10072.86520078126</v>
+        <v>9546.6869690003168</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="7"/>
@@ -1303,12 +1302,12 @@
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="10">
-        <v>45412</v>
+        <v>45382</v>
       </c>
       <c r="B54" s="7">
-        <v>9874.8838561473312</v>
+        <v>10072.86520078126</v>
       </c>
       <c r="C54" s="10"/>
       <c r="D54" s="7"/>
@@ -1320,12 +1319,12 @@
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="10">
-        <v>45443</v>
+        <v>45412</v>
       </c>
       <c r="B55" s="7">
-        <v>9582.6</v>
+        <v>9874.8838561473312</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="7"/>
@@ -1337,12 +1336,12 @@
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="10">
-        <v>45473</v>
+        <v>45443</v>
       </c>
       <c r="B56" s="7">
-        <v>13313.671420838193</v>
+        <v>9582.6</v>
       </c>
       <c r="C56" s="10"/>
       <c r="D56" s="7"/>
@@ -1354,12 +1353,12 @@
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="10">
-        <v>45504</v>
+        <v>45473</v>
       </c>
       <c r="B57" s="7">
-        <v>13431.891383190006</v>
+        <v>13313.671420838193</v>
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="7"/>
@@ -1371,12 +1370,12 @@
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="10">
-        <v>45535</v>
+        <v>45504</v>
       </c>
       <c r="B58" s="7">
-        <v>11558.85</v>
+        <v>13431.891383190006</v>
       </c>
       <c r="C58" s="10"/>
       <c r="D58" s="7"/>
@@ -1388,12 +1387,12 @@
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="10">
-        <v>45565</v>
+        <v>45535</v>
       </c>
       <c r="B59" s="7">
-        <v>10153.379999999999</v>
+        <v>11558.85</v>
       </c>
       <c r="C59" s="10"/>
       <c r="D59" s="7"/>
@@ -1405,15 +1404,15 @@
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="10">
-        <v>45596</v>
+        <v>45565</v>
       </c>
       <c r="B60" s="7">
-        <v>9348.3390886612633</v>
+        <v>10153.379999999999</v>
       </c>
       <c r="C60" s="10"/>
-      <c r="D60" s="1"/>
+      <c r="D60" s="7"/>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
@@ -1422,15 +1421,15 @@
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="10">
-        <v>45626</v>
+        <v>45596</v>
       </c>
       <c r="B61" s="7">
-        <v>10429.950000000001</v>
+        <v>9348.3390886612633</v>
       </c>
       <c r="C61" s="10"/>
-      <c r="D61" s="7"/>
+      <c r="D61" s="1"/>
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
@@ -1439,14 +1438,14 @@
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="10">
-        <v>45657</v>
+        <v>45626</v>
       </c>
       <c r="B62" s="7">
-        <v>12709.7</v>
-      </c>
-      <c r="C62" s="16"/>
+        <v>10429.950000000001</v>
+      </c>
+      <c r="C62" s="10"/>
       <c r="D62" s="7"/>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
@@ -1456,14 +1455,14 @@
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="10">
-        <v>45688</v>
+        <v>45657</v>
       </c>
       <c r="B63" s="7">
-        <v>14484.61</v>
-      </c>
-      <c r="C63" s="10"/>
+        <v>12709.7</v>
+      </c>
+      <c r="C63" s="16"/>
       <c r="D63" s="7"/>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
@@ -1473,15 +1472,15 @@
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" s="10">
-        <v>45716</v>
+        <v>45688</v>
       </c>
       <c r="B64" s="7">
-        <v>12523.542647105076</v>
+        <v>14484.61</v>
       </c>
       <c r="C64" s="10"/>
-      <c r="D64" s="1"/>
+      <c r="D64" s="7"/>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
@@ -1490,15 +1489,15 @@
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A65" s="15">
-        <v>45747</v>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A65" s="10">
+        <v>45716</v>
       </c>
       <c r="B65" s="7">
-        <v>11731.849510343653</v>
+        <v>12523.542647105076</v>
       </c>
       <c r="C65" s="10"/>
-      <c r="D65" s="7"/>
+      <c r="D65" s="1"/>
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
@@ -1507,12 +1506,12 @@
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A66" s="10">
-        <v>45777</v>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A66" s="15">
+        <v>45747</v>
       </c>
       <c r="B66" s="7">
-        <v>10591.553241003245</v>
+        <v>11731.849510343653</v>
       </c>
       <c r="C66" s="10"/>
       <c r="D66" s="7"/>
@@ -1524,12 +1523,12 @@
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" s="10">
-        <v>45808</v>
+        <v>45777</v>
       </c>
       <c r="B67" s="7">
-        <v>9922.4680665252672</v>
+        <v>10591.553241003245</v>
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="7"/>
@@ -1541,15 +1540,15 @@
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" s="10">
-        <v>45838</v>
+        <v>45808</v>
       </c>
       <c r="B68" s="7">
-        <v>9409.0667305531842</v>
+        <v>9922.4680665252672</v>
       </c>
       <c r="C68" s="10"/>
-      <c r="D68" s="1"/>
+      <c r="D68" s="7"/>
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
@@ -1558,15 +1557,15 @@
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" s="10">
-        <v>45869</v>
+        <v>45838</v>
       </c>
       <c r="B69" s="7">
-        <v>9384.6811267681933</v>
+        <v>9409.0667305531842</v>
       </c>
       <c r="C69" s="10"/>
-      <c r="D69" s="7"/>
+      <c r="D69" s="1"/>
       <c r="E69" s="2"/>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
@@ -1575,12 +1574,12 @@
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" s="10">
-        <v>45900</v>
+        <v>45869</v>
       </c>
       <c r="B70" s="7">
-        <v>6686.0673348374312</v>
+        <v>9384.6811267681933</v>
       </c>
       <c r="C70" s="10"/>
       <c r="D70" s="7"/>
@@ -1592,12 +1591,12 @@
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" s="10">
-        <v>45930</v>
+        <v>45900</v>
       </c>
       <c r="B71" s="7">
-        <v>6857</v>
+        <v>6686.0673348374312</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="7"/>
@@ -1609,12 +1608,12 @@
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" s="10">
-        <v>45961</v>
+        <v>45930</v>
       </c>
       <c r="B72" s="7">
-        <v>7857.6643179510265</v>
+        <v>6857</v>
       </c>
       <c r="C72" s="10"/>
       <c r="D72" s="7"/>
@@ -1626,12 +1625,12 @@
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" s="10">
-        <v>45991</v>
+        <v>45961</v>
       </c>
       <c r="B73" s="7">
-        <v>7189.52</v>
+        <v>7857.6643179510265</v>
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="7"/>
@@ -1643,15 +1642,15 @@
       <c r="J73" s="2"/>
       <c r="K73" s="2"/>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" s="10">
-        <v>46022</v>
+        <v>45991</v>
       </c>
       <c r="B74" s="7">
-        <v>6210.4203163321936</v>
+        <v>7189.52</v>
       </c>
       <c r="C74" s="10"/>
-      <c r="D74" s="1"/>
+      <c r="D74" s="7"/>
       <c r="E74" s="2"/>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
@@ -1660,12 +1659,12 @@
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" s="10">
-        <v>46053</v>
+        <v>46022</v>
       </c>
       <c r="B75" s="7">
-        <v>5551.5682809355858</v>
+        <v>6210.4203163321936</v>
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="1"/>
@@ -1677,14 +1676,15 @@
       <c r="J75" s="2"/>
       <c r="K75" s="2"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" s="10">
-        <v>46081</v>
+        <v>46053</v>
       </c>
       <c r="B76" s="7">
-        <v>5968.5038551168427</v>
+        <v>5551.5682809355858</v>
       </c>
       <c r="C76" s="10"/>
+      <c r="D76" s="1"/>
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
@@ -1693,13 +1693,14 @@
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" s="10">
-        <v>46112</v>
+        <v>46081</v>
       </c>
       <c r="B77" s="7">
-        <v>6358.7504043637091</v>
-      </c>
+        <v>5968.5038551168427</v>
+      </c>
+      <c r="C77" s="10"/>
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
@@ -1708,12 +1709,12 @@
       <c r="J77" s="2"/>
       <c r="K77" s="2"/>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" s="10">
-        <v>46142</v>
+        <v>46112</v>
       </c>
       <c r="B78" s="7">
-        <v>6072.5891264595048</v>
+        <v>6358.7504043637091</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
@@ -1723,12 +1724,12 @@
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" s="10">
-        <v>46173</v>
+        <v>46142</v>
       </c>
       <c r="B79" s="7">
-        <v>5951.4636637017702</v>
+        <v>6072.5891264595048</v>
       </c>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
@@ -1738,12 +1739,12 @@
       <c r="J79" s="2"/>
       <c r="K79" s="2"/>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" s="10">
-        <v>46203</v>
+        <v>46173</v>
       </c>
       <c r="B80" s="7">
-        <v>6787.0405811540904</v>
+        <v>5951.4636637017702</v>
       </c>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
@@ -1753,12 +1754,12 @@
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" s="10">
-        <v>46234</v>
+        <v>46203</v>
       </c>
       <c r="B81" s="7">
-        <v>5428.095078319494</v>
+        <v>6787.0405811540904</v>
       </c>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
@@ -1768,12 +1769,12 @@
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" s="10">
-        <v>46265</v>
+        <v>46234</v>
       </c>
       <c r="B82" s="7">
-        <v>5611.7970995836176</v>
+        <v>5428.095078319494</v>
       </c>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
@@ -1783,8 +1784,13 @@
       <c r="J82" s="2"/>
       <c r="K82" s="2"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B83" s="7"/>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A83" s="10">
+        <v>46265</v>
+      </c>
+      <c r="B83" s="7">
+        <v>5611.7970995836176</v>
+      </c>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
@@ -1793,11 +1799,13 @@
       <c r="J83" s="2"/>
       <c r="K83" s="2"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A84" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B84" s="7"/>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A84" s="10">
+        <v>46295</v>
+      </c>
+      <c r="B84" s="7">
+        <v>5187.0964722611998</v>
+      </c>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
@@ -1806,8 +1814,8 @@
       <c r="J84" s="2"/>
       <c r="K84" s="2"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A85" s="10"/>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B85" s="7"/>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
@@ -1816,8 +1824,10 @@
       <c r="J85" s="2"/>
       <c r="K85" s="2"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A86" s="10"/>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A86" s="16" t="s">
+        <v>5</v>
+      </c>
       <c r="B86" s="7"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
@@ -1827,9 +1837,8 @@
       <c r="J86" s="2"/>
       <c r="K86" s="2"/>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" s="10"/>
-      <c r="B87" s="7"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
@@ -1838,7 +1847,7 @@
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" s="10"/>
       <c r="B88" s="7"/>
       <c r="E88" s="2"/>
@@ -1849,8 +1858,9 @@
       <c r="J88" s="2"/>
       <c r="K88" s="2"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" s="10"/>
+      <c r="B89" s="7"/>
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
@@ -1859,8 +1869,9 @@
       <c r="J89" s="2"/>
       <c r="K89" s="2"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" s="10"/>
+      <c r="B90" s="7"/>
       <c r="E90" s="2"/>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
@@ -1869,7 +1880,8 @@
       <c r="J90" s="2"/>
       <c r="K90" s="2"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A91" s="10"/>
       <c r="E91" s="2"/>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
@@ -1878,8 +1890,9 @@
       <c r="J91" s="2"/>
       <c r="K91" s="2"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E92" s="11"/>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A92" s="10"/>
+      <c r="E92" s="2"/>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
@@ -1887,8 +1900,8 @@
       <c r="J92" s="2"/>
       <c r="K92" s="2"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="E93" s="11"/>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="E93" s="2"/>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
@@ -1896,7 +1909,7 @@
       <c r="J93" s="2"/>
       <c r="K93" s="2"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E94" s="11"/>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
@@ -1905,7 +1918,7 @@
       <c r="J94" s="2"/>
       <c r="K94" s="2"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E95" s="11"/>
       <c r="F95" s="2"/>
       <c r="G95" s="2"/>
@@ -1914,7 +1927,7 @@
       <c r="J95" s="2"/>
       <c r="K95" s="2"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E96" s="11"/>
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
@@ -1923,7 +1936,7 @@
       <c r="J96" s="2"/>
       <c r="K96" s="2"/>
     </row>
-    <row r="97" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E97" s="11"/>
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
@@ -1932,7 +1945,7 @@
       <c r="J97" s="2"/>
       <c r="K97" s="2"/>
     </row>
-    <row r="98" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E98" s="11"/>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
@@ -1941,7 +1954,7 @@
       <c r="J98" s="2"/>
       <c r="K98" s="2"/>
     </row>
-    <row r="99" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E99" s="11"/>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
@@ -1950,7 +1963,7 @@
       <c r="J99" s="2"/>
       <c r="K99" s="2"/>
     </row>
-    <row r="100" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E100" s="11"/>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
@@ -1959,7 +1972,7 @@
       <c r="J100" s="2"/>
       <c r="K100" s="2"/>
     </row>
-    <row r="101" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E101" s="11"/>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
@@ -1968,7 +1981,7 @@
       <c r="J101" s="2"/>
       <c r="K101" s="2"/>
     </row>
-    <row r="102" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E102" s="11"/>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
@@ -1977,7 +1990,7 @@
       <c r="J102" s="2"/>
       <c r="K102" s="2"/>
     </row>
-    <row r="103" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E103" s="11"/>
       <c r="F103" s="2"/>
       <c r="G103" s="2"/>
@@ -1986,7 +1999,7 @@
       <c r="J103" s="2"/>
       <c r="K103" s="2"/>
     </row>
-    <row r="104" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E104" s="11"/>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
@@ -1995,7 +2008,7 @@
       <c r="J104" s="2"/>
       <c r="K104" s="2"/>
     </row>
-    <row r="105" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E105" s="11"/>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
@@ -2004,7 +2017,7 @@
       <c r="J105" s="2"/>
       <c r="K105" s="2"/>
     </row>
-    <row r="106" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E106" s="11"/>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
@@ -2013,7 +2026,7 @@
       <c r="J106" s="2"/>
       <c r="K106" s="2"/>
     </row>
-    <row r="107" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E107" s="11"/>
       <c r="F107" s="2"/>
       <c r="G107" s="2"/>
@@ -2022,7 +2035,7 @@
       <c r="J107" s="2"/>
       <c r="K107" s="2"/>
     </row>
-    <row r="108" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E108" s="11"/>
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
@@ -2031,7 +2044,7 @@
       <c r="J108" s="2"/>
       <c r="K108" s="2"/>
     </row>
-    <row r="109" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E109" s="11"/>
       <c r="F109" s="2"/>
       <c r="G109" s="2"/>
@@ -2040,7 +2053,7 @@
       <c r="J109" s="2"/>
       <c r="K109" s="2"/>
     </row>
-    <row r="110" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E110" s="11"/>
       <c r="F110" s="2"/>
       <c r="G110" s="2"/>
@@ -2049,7 +2062,7 @@
       <c r="J110" s="2"/>
       <c r="K110" s="2"/>
     </row>
-    <row r="111" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E111" s="11"/>
       <c r="F111" s="2"/>
       <c r="G111" s="2"/>
@@ -2058,7 +2071,7 @@
       <c r="J111" s="2"/>
       <c r="K111" s="2"/>
     </row>
-    <row r="112" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E112" s="11"/>
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
@@ -2067,7 +2080,7 @@
       <c r="J112" s="2"/>
       <c r="K112" s="2"/>
     </row>
-    <row r="113" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E113" s="11"/>
       <c r="F113" s="2"/>
       <c r="G113" s="2"/>
@@ -2076,7 +2089,7 @@
       <c r="J113" s="2"/>
       <c r="K113" s="2"/>
     </row>
-    <row r="114" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E114" s="11"/>
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
@@ -2085,7 +2098,7 @@
       <c r="J114" s="2"/>
       <c r="K114" s="2"/>
     </row>
-    <row r="115" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E115" s="11"/>
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
@@ -2094,7 +2107,7 @@
       <c r="J115" s="2"/>
       <c r="K115" s="2"/>
     </row>
-    <row r="116" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E116" s="11"/>
       <c r="F116" s="2"/>
       <c r="G116" s="2"/>
@@ -2103,8 +2116,8 @@
       <c r="J116" s="2"/>
       <c r="K116" s="2"/>
     </row>
-    <row r="117" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E117" s="2"/>
+    <row r="117" spans="5:11" x14ac:dyDescent="0.35">
+      <c r="E117" s="11"/>
       <c r="F117" s="2"/>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
@@ -2112,8 +2125,8 @@
       <c r="J117" s="2"/>
       <c r="K117" s="2"/>
     </row>
-    <row r="118" spans="5:11" x14ac:dyDescent="0.25">
-      <c r="E118" s="2"/>
+    <row r="118" spans="5:11" x14ac:dyDescent="0.35">
+      <c r="E118" s="11"/>
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
@@ -2121,7 +2134,7 @@
       <c r="J118" s="2"/>
       <c r="K118" s="2"/>
     </row>
-    <row r="119" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E119" s="2"/>
       <c r="F119" s="2"/>
       <c r="G119" s="2"/>
@@ -2130,7 +2143,7 @@
       <c r="J119" s="2"/>
       <c r="K119" s="2"/>
     </row>
-    <row r="120" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E120" s="2"/>
       <c r="F120" s="2"/>
       <c r="G120" s="2"/>
@@ -2139,7 +2152,7 @@
       <c r="J120" s="2"/>
       <c r="K120" s="2"/>
     </row>
-    <row r="121" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E121" s="2"/>
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
@@ -2148,7 +2161,7 @@
       <c r="J121" s="2"/>
       <c r="K121" s="2"/>
     </row>
-    <row r="122" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E122" s="2"/>
       <c r="F122" s="2"/>
       <c r="G122" s="2"/>
@@ -2157,7 +2170,7 @@
       <c r="J122" s="2"/>
       <c r="K122" s="2"/>
     </row>
-    <row r="123" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E123" s="2"/>
       <c r="F123" s="2"/>
       <c r="G123" s="2"/>
@@ -2166,7 +2179,7 @@
       <c r="J123" s="2"/>
       <c r="K123" s="2"/>
     </row>
-    <row r="124" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E124" s="2"/>
       <c r="F124" s="2"/>
       <c r="G124" s="2"/>
@@ -2175,7 +2188,7 @@
       <c r="J124" s="2"/>
       <c r="K124" s="2"/>
     </row>
-    <row r="125" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E125" s="2"/>
       <c r="F125" s="2"/>
       <c r="G125" s="2"/>
@@ -2184,7 +2197,7 @@
       <c r="J125" s="2"/>
       <c r="K125" s="2"/>
     </row>
-    <row r="126" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E126" s="2"/>
       <c r="F126" s="2"/>
       <c r="G126" s="2"/>
@@ -2193,7 +2206,7 @@
       <c r="J126" s="2"/>
       <c r="K126" s="2"/>
     </row>
-    <row r="127" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E127" s="2"/>
       <c r="F127" s="2"/>
       <c r="G127" s="2"/>
@@ -2202,7 +2215,7 @@
       <c r="J127" s="2"/>
       <c r="K127" s="2"/>
     </row>
-    <row r="128" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E128" s="2"/>
       <c r="F128" s="2"/>
       <c r="G128" s="2"/>
@@ -2211,7 +2224,7 @@
       <c r="J128" s="2"/>
       <c r="K128" s="2"/>
     </row>
-    <row r="129" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E129" s="2"/>
       <c r="F129" s="2"/>
       <c r="G129" s="2"/>
@@ -2220,7 +2233,7 @@
       <c r="J129" s="2"/>
       <c r="K129" s="2"/>
     </row>
-    <row r="130" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E130" s="2"/>
       <c r="F130" s="2"/>
       <c r="G130" s="2"/>
@@ -2229,7 +2242,7 @@
       <c r="J130" s="2"/>
       <c r="K130" s="2"/>
     </row>
-    <row r="131" spans="5:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="5:11" x14ac:dyDescent="0.35">
       <c r="E131" s="2"/>
       <c r="F131" s="2"/>
       <c r="G131" s="2"/>
@@ -2238,6 +2251,24 @@
       <c r="J131" s="2"/>
       <c r="K131" s="2"/>
     </row>
+    <row r="132" spans="5:11" x14ac:dyDescent="0.35">
+      <c r="E132" s="2"/>
+      <c r="F132" s="2"/>
+      <c r="G132" s="2"/>
+      <c r="H132" s="2"/>
+      <c r="I132" s="2"/>
+      <c r="J132" s="2"/>
+      <c r="K132" s="2"/>
+    </row>
+    <row r="133" spans="5:11" x14ac:dyDescent="0.35">
+      <c r="E133" s="2"/>
+      <c r="F133" s="2"/>
+      <c r="G133" s="2"/>
+      <c r="H133" s="2"/>
+      <c r="I133" s="2"/>
+      <c r="J133" s="2"/>
+      <c r="K133" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2245,15 +2276,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010029EFE90E92722F4EB0850C4107E61AFD" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d64f42a1a065c4567c2c4a54e2f44f2a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c5dd58c6-0651-4634-b1fc-70af4a74b2bb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5c8912e392fdf01a21952510fd4c13b5" ns2:_="">
     <xsd:import namespace="c5dd58c6-0651-4634-b1fc-70af4a74b2bb"/>
@@ -2397,21 +2419,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65ECF0E8-C5CC-4AAD-91AC-F4300C517343}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB4E957D-89E0-4998-82E2-A565733AC20C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2429,18 +2452,26 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7497209-7BE2-4958-B95F-E5461CF73321}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c5dd58c6-0651-4634-b1fc-70af4a74b2bb"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="c5dd58c6-0651-4634-b1fc-70af4a74b2bb"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65ECF0E8-C5CC-4AAD-91AC-F4300C517343}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>